<commit_message>
Added change file upload-merge (upload-update) service where admin/superadmin can update any item/category/service or add new item/category/service to existing data
</commit_message>
<xml_diff>
--- a/uploads/menu_data_2.xlsx
+++ b/uploads/menu_data_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4fdae77fc648ca8d/Desktop/SAAS_MENU/saas-menu-app-backend/uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="8_{A2AF0A05-CFD6-44AF-B283-622CE488AF25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{540355B0-BC6B-4FBA-9929-863DCFF22BE3}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="8_{A2AF0A05-CFD6-44AF-B283-622CE488AF25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99F8C6F3-B3DB-4064-A3FA-87B344A20DBC}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -335,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -343,15 +343,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -367,6 +358,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -727,10 +722,10 @@
       <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" t="s">
         <v>29</v>
       </c>
     </row>
@@ -738,10 +733,10 @@
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" t="s">
         <v>30</v>
       </c>
     </row>
@@ -749,10 +744,10 @@
       <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" t="s">
         <v>31</v>
       </c>
     </row>
@@ -760,10 +755,10 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" t="s">
         <v>28</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" t="s">
         <v>32</v>
       </c>
     </row>
@@ -774,10 +769,10 @@
       <c r="B6" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" t="s">
         <v>41</v>
       </c>
     </row>
@@ -785,13 +780,13 @@
       <c r="A7" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" t="s">
         <v>42</v>
       </c>
     </row>
@@ -802,10 +797,10 @@
       <c r="B8" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" t="s">
         <v>43</v>
       </c>
     </row>
@@ -813,13 +808,13 @@
       <c r="A9" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" t="s">
         <v>44</v>
       </c>
     </row>
@@ -830,10 +825,10 @@
       <c r="B10" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" t="s">
         <v>45</v>
       </c>
     </row>
@@ -841,13 +836,13 @@
       <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" t="s">
         <v>38</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" t="s">
         <v>46</v>
       </c>
     </row>
@@ -858,10 +853,10 @@
       <c r="B12" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" t="s">
         <v>47</v>
       </c>
     </row>
@@ -869,13 +864,13 @@
       <c r="A13" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" t="s">
         <v>40</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" t="s">
         <v>48</v>
       </c>
     </row>
@@ -883,47 +878,46 @@
       <c r="A14" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" t="s">
         <v>58</v>
       </c>
-      <c r="F14" s="10">
-        <v>450</v>
-      </c>
-      <c r="G14" s="11" t="s">
+      <c r="F14">
+        <v>550</v>
+      </c>
+      <c r="G14" t="s">
         <v>12</v>
       </c>
-      <c r="H14" s="11" t="s">
+      <c r="H14" t="s">
         <v>13</v>
       </c>
-      <c r="I14" s="11">
+      <c r="I14">
         <v>600</v>
       </c>
-      <c r="J14" s="11">
+      <c r="J14">
         <v>50</v>
       </c>
-      <c r="K14" s="11">
+      <c r="K14">
         <v>5</v>
       </c>
-      <c r="L14" s="11">
+      <c r="L14">
         <v>40</v>
       </c>
-      <c r="M14" s="11" t="s">
+      <c r="M14" t="s">
         <v>67</v>
       </c>
-      <c r="N14" s="11" t="s">
+      <c r="N14" t="s">
         <v>68</v>
       </c>
-      <c r="O14" s="11"/>
-      <c r="P14" s="11" t="b">
+      <c r="P14" t="b">
         <v>1</v>
       </c>
-      <c r="Q14" s="11" t="b">
+      <c r="Q14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -931,47 +925,46 @@
       <c r="A15" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" t="s">
         <v>33</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" t="s">
         <v>50</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" t="s">
         <v>59</v>
       </c>
-      <c r="F15" s="10">
+      <c r="F15">
         <v>500</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="G15" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="11" t="s">
+      <c r="H15" t="s">
         <v>13</v>
       </c>
-      <c r="I15" s="11">
+      <c r="I15">
         <v>700</v>
       </c>
-      <c r="J15" s="11">
+      <c r="J15">
         <v>55</v>
       </c>
-      <c r="K15" s="11">
+      <c r="K15">
         <v>3</v>
       </c>
-      <c r="L15" s="11">
+      <c r="L15">
         <v>45</v>
       </c>
-      <c r="M15" s="11" t="s">
+      <c r="M15" t="s">
         <v>67</v>
       </c>
-      <c r="N15" s="11" t="s">
+      <c r="N15" t="s">
         <v>69</v>
       </c>
-      <c r="O15" s="11"/>
-      <c r="P15" s="11" t="b">
+      <c r="P15" t="b">
         <v>1</v>
       </c>
-      <c r="Q15" s="11" t="b">
+      <c r="Q15" t="b">
         <v>0</v>
       </c>
     </row>
@@ -979,47 +972,46 @@
       <c r="A16" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" t="s">
         <v>51</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" t="s">
         <v>60</v>
       </c>
-      <c r="F16" s="10">
+      <c r="F16">
         <v>400</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" t="s">
         <v>12</v>
       </c>
-      <c r="H16" s="11" t="s">
+      <c r="H16" t="s">
         <v>13</v>
       </c>
-      <c r="I16" s="11">
+      <c r="I16">
         <v>550</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J16">
         <v>45</v>
       </c>
-      <c r="K16" s="11">
+      <c r="K16">
         <v>6</v>
       </c>
-      <c r="L16" s="11">
+      <c r="L16">
         <v>30</v>
       </c>
-      <c r="M16" s="11" t="s">
+      <c r="M16" t="s">
         <v>67</v>
       </c>
-      <c r="N16" s="11" t="s">
+      <c r="N16" t="s">
         <v>70</v>
       </c>
-      <c r="O16" s="11"/>
-      <c r="P16" s="11" t="b">
+      <c r="P16" t="b">
         <v>1</v>
       </c>
-      <c r="Q16" s="11" t="b">
+      <c r="Q16" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1027,47 +1019,46 @@
       <c r="A17" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" t="s">
         <v>35</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" t="s">
         <v>52</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" t="s">
         <v>61</v>
       </c>
-      <c r="F17" s="10">
+      <c r="F17">
         <v>250</v>
       </c>
-      <c r="G17" s="11" t="s">
+      <c r="G17" t="s">
         <v>11</v>
       </c>
-      <c r="H17" s="11" t="s">
+      <c r="H17" t="s">
         <v>13</v>
       </c>
-      <c r="I17" s="11">
+      <c r="I17">
         <v>450</v>
       </c>
-      <c r="J17" s="11">
+      <c r="J17">
         <v>12</v>
       </c>
-      <c r="K17" s="11">
+      <c r="K17">
         <v>60</v>
       </c>
-      <c r="L17" s="11">
+      <c r="L17">
         <v>20</v>
       </c>
-      <c r="M17" s="11" t="s">
+      <c r="M17" t="s">
         <v>71</v>
       </c>
-      <c r="N17" s="11" t="s">
+      <c r="N17" t="s">
         <v>72</v>
       </c>
-      <c r="O17" s="11"/>
-      <c r="P17" s="11" t="b">
+      <c r="P17" t="b">
         <v>1</v>
       </c>
-      <c r="Q17" s="11" t="b">
+      <c r="Q17" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1075,47 +1066,46 @@
       <c r="A18" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" t="s">
         <v>53</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="E18" t="s">
         <v>62</v>
       </c>
-      <c r="F18" s="10">
+      <c r="F18">
         <v>300</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" t="s">
         <v>11</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="H18" t="s">
         <v>14</v>
       </c>
-      <c r="I18" s="11">
+      <c r="I18">
         <v>600</v>
       </c>
-      <c r="J18" s="11">
+      <c r="J18">
         <v>15</v>
       </c>
-      <c r="K18" s="11">
+      <c r="K18">
         <v>80</v>
       </c>
-      <c r="L18" s="11">
+      <c r="L18">
         <v>20</v>
       </c>
-      <c r="M18" s="11" t="s">
+      <c r="M18" t="s">
         <v>73</v>
       </c>
-      <c r="N18" s="11" t="s">
+      <c r="N18" t="s">
         <v>74</v>
       </c>
-      <c r="O18" s="11"/>
-      <c r="P18" s="11" t="b">
+      <c r="P18" t="b">
         <v>1</v>
       </c>
-      <c r="Q18" s="11" t="b">
+      <c r="Q18" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1123,47 +1113,46 @@
       <c r="A19" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" t="s">
         <v>54</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" t="s">
         <v>63</v>
       </c>
-      <c r="F19" s="10">
+      <c r="F19">
         <v>150</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="G19" t="s">
         <v>11</v>
       </c>
-      <c r="H19" s="11" t="s">
+      <c r="H19" t="s">
         <v>15</v>
       </c>
-      <c r="I19" s="11">
+      <c r="I19">
         <v>200</v>
       </c>
-      <c r="J19" s="11">
+      <c r="J19">
         <v>5</v>
       </c>
-      <c r="K19" s="11">
+      <c r="K19">
         <v>40</v>
       </c>
-      <c r="L19" s="11">
+      <c r="L19">
         <v>5</v>
       </c>
-      <c r="M19" s="11" t="s">
+      <c r="M19" t="s">
         <v>67</v>
       </c>
-      <c r="N19" s="11" t="s">
+      <c r="N19" t="s">
         <v>75</v>
       </c>
-      <c r="O19" s="11"/>
-      <c r="P19" s="11" t="b">
+      <c r="P19" t="b">
         <v>1</v>
       </c>
-      <c r="Q19" s="11" t="b">
+      <c r="Q19" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1171,47 +1160,46 @@
       <c r="A20" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" t="s">
         <v>38</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" t="s">
         <v>55</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E20" t="s">
         <v>64</v>
       </c>
-      <c r="F20" s="10">
+      <c r="F20">
         <v>180</v>
       </c>
-      <c r="G20" s="11" t="s">
+      <c r="G20" t="s">
         <v>11</v>
       </c>
-      <c r="H20" s="11" t="s">
+      <c r="H20" t="s">
         <v>76</v>
       </c>
-      <c r="I20" s="11">
+      <c r="I20">
         <v>350</v>
       </c>
-      <c r="J20" s="11">
+      <c r="J20">
         <v>15</v>
       </c>
-      <c r="K20" s="11">
+      <c r="K20">
         <v>50</v>
       </c>
-      <c r="L20" s="11">
+      <c r="L20">
         <v>10</v>
       </c>
-      <c r="M20" s="11" t="s">
+      <c r="M20" t="s">
         <v>67</v>
       </c>
-      <c r="N20" s="11" t="s">
+      <c r="N20" t="s">
         <v>77</v>
       </c>
-      <c r="O20" s="11"/>
-      <c r="P20" s="11" t="b">
+      <c r="P20" t="b">
         <v>1</v>
       </c>
-      <c r="Q20" s="11" t="b">
+      <c r="Q20" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1219,47 +1207,46 @@
       <c r="A21" t="s">
         <v>10</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" t="s">
         <v>39</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" t="s">
         <v>56</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" t="s">
         <v>65</v>
       </c>
-      <c r="F21" s="10">
+      <c r="F21">
         <v>400</v>
       </c>
-      <c r="G21" s="11" t="s">
+      <c r="G21" t="s">
         <v>12</v>
       </c>
-      <c r="H21" s="11" t="s">
+      <c r="H21" t="s">
         <v>13</v>
       </c>
-      <c r="I21" s="11">
+      <c r="I21">
         <v>500</v>
       </c>
-      <c r="J21" s="11">
+      <c r="J21">
         <v>40</v>
       </c>
-      <c r="K21" s="11">
+      <c r="K21">
         <v>3</v>
       </c>
-      <c r="L21" s="11">
+      <c r="L21">
         <v>25</v>
       </c>
-      <c r="M21" s="11" t="s">
+      <c r="M21" t="s">
         <v>78</v>
       </c>
-      <c r="N21" s="11" t="s">
+      <c r="N21" t="s">
         <v>79</v>
       </c>
-      <c r="O21" s="11"/>
-      <c r="P21" s="11" t="b">
+      <c r="P21" t="b">
         <v>1</v>
       </c>
-      <c r="Q21" s="11" t="b">
+      <c r="Q21" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1267,47 +1254,46 @@
       <c r="A22" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" t="s">
         <v>40</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" t="s">
         <v>57</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="E22" t="s">
         <v>66</v>
       </c>
-      <c r="F22" s="10">
+      <c r="F22">
         <v>600</v>
       </c>
-      <c r="G22" s="11" t="s">
+      <c r="G22" t="s">
         <v>12</v>
       </c>
-      <c r="H22" s="11" t="s">
+      <c r="H22" t="s">
         <v>14</v>
       </c>
-      <c r="I22" s="11">
+      <c r="I22">
         <v>750</v>
       </c>
-      <c r="J22" s="11">
+      <c r="J22">
         <v>60</v>
       </c>
-      <c r="K22" s="11">
+      <c r="K22">
         <v>5</v>
       </c>
-      <c r="L22" s="11">
+      <c r="L22">
         <v>35</v>
       </c>
-      <c r="M22" s="11" t="s">
+      <c r="M22" t="s">
         <v>80</v>
       </c>
-      <c r="N22" s="11" t="s">
+      <c r="N22" t="s">
         <v>81</v>
       </c>
-      <c r="O22" s="11"/>
-      <c r="P22" s="11" t="b">
+      <c r="P22" t="b">
         <v>1</v>
       </c>
-      <c r="Q22" s="11" t="b">
+      <c r="Q22" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added audit logs for tracking all the changes
</commit_message>
<xml_diff>
--- a/uploads/menu_data_2.xlsx
+++ b/uploads/menu_data_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4fdae77fc648ca8d/Desktop/SAAS_MENU/saas-menu-app-backend/uploads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="8_{A2AF0A05-CFD6-44AF-B283-622CE488AF25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99F8C6F3-B3DB-4064-A3FA-87B344A20DBC}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="8_{A2AF0A05-CFD6-44AF-B283-622CE488AF25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8F8D49E-5F51-495D-8CFA-52B39BA30D9B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="89">
   <si>
     <t>type</t>
   </si>
@@ -120,18 +120,12 @@
     <t>Seafood Grill</t>
   </si>
   <si>
-    <t>Fine dining with premium steaks</t>
-  </si>
-  <si>
     <t>Authentic Italian pasta and pizza</t>
   </si>
   <si>
     <t>Plant-based food and drinks</t>
   </si>
   <si>
-    <t>Fresh seafood, grilled to perfection</t>
-  </si>
-  <si>
     <t>Grilled Steaks</t>
   </si>
   <si>
@@ -277,6 +271,33 @@
   </si>
   <si>
     <t>Shrimp, Lobster, Garlic</t>
+  </si>
+  <si>
+    <t>Serves 4</t>
+  </si>
+  <si>
+    <t>Fine dining with premium steaks and fishes</t>
+  </si>
+  <si>
+    <t>New Service</t>
+  </si>
+  <si>
+    <t>New Category</t>
+  </si>
+  <si>
+    <t>New Item</t>
+  </si>
+  <si>
+    <t>Fresh seafood, grilled to perfection made</t>
+  </si>
+  <si>
+    <t>New Service 2</t>
+  </si>
+  <si>
+    <t>New Category 2</t>
+  </si>
+  <si>
+    <t>New Item 2</t>
   </si>
 </sst>
 </file>
@@ -651,7 +672,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R22"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
@@ -726,7 +747,7 @@
         <v>25</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
@@ -737,7 +758,7 @@
         <v>26</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
@@ -748,7 +769,7 @@
         <v>27</v>
       </c>
       <c r="E4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
@@ -759,7 +780,7 @@
         <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
@@ -770,10 +791,10 @@
         <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
@@ -784,10 +805,10 @@
         <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
@@ -798,10 +819,10 @@
         <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
@@ -812,10 +833,10 @@
         <v>26</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
@@ -826,10 +847,10 @@
         <v>27</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
@@ -840,10 +861,10 @@
         <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
@@ -854,10 +875,10 @@
         <v>28</v>
       </c>
       <c r="D12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E12" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
@@ -868,10 +889,10 @@
         <v>28</v>
       </c>
       <c r="D13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E13" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
@@ -879,22 +900,22 @@
         <v>10</v>
       </c>
       <c r="C14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D14" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E14" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F14">
-        <v>550</v>
+        <v>350</v>
       </c>
       <c r="G14" t="s">
         <v>12</v>
       </c>
       <c r="H14" t="s">
-        <v>13</v>
+        <v>80</v>
       </c>
       <c r="I14">
         <v>600</v>
@@ -909,10 +930,10 @@
         <v>40</v>
       </c>
       <c r="M14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N14" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="P14" t="b">
         <v>1</v>
@@ -926,13 +947,13 @@
         <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D15" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E15" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F15">
         <v>500</v>
@@ -956,10 +977,10 @@
         <v>45</v>
       </c>
       <c r="M15" t="s">
+        <v>65</v>
+      </c>
+      <c r="N15" t="s">
         <v>67</v>
-      </c>
-      <c r="N15" t="s">
-        <v>69</v>
       </c>
       <c r="P15" t="b">
         <v>1</v>
@@ -973,13 +994,13 @@
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D16" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E16" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F16">
         <v>400</v>
@@ -1003,10 +1024,10 @@
         <v>30</v>
       </c>
       <c r="M16" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N16" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="P16" t="b">
         <v>1</v>
@@ -1020,13 +1041,13 @@
         <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D17" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F17">
         <v>250</v>
@@ -1050,10 +1071,10 @@
         <v>20</v>
       </c>
       <c r="M17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N17" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="P17" t="b">
         <v>1</v>
@@ -1067,13 +1088,13 @@
         <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D18" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F18">
         <v>300</v>
@@ -1082,10 +1103,10 @@
         <v>11</v>
       </c>
       <c r="H18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I18">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="J18">
         <v>15</v>
@@ -1097,10 +1118,10 @@
         <v>20</v>
       </c>
       <c r="M18" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="N18" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="P18" t="b">
         <v>1</v>
@@ -1114,13 +1135,13 @@
         <v>10</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D19" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E19" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F19">
         <v>150</v>
@@ -1144,10 +1165,10 @@
         <v>5</v>
       </c>
       <c r="M19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N19" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="P19" t="b">
         <v>1</v>
@@ -1161,22 +1182,22 @@
         <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D20" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E20" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F20">
-        <v>180</v>
+        <v>280</v>
       </c>
       <c r="G20" t="s">
         <v>11</v>
       </c>
       <c r="H20" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I20">
         <v>350</v>
@@ -1191,10 +1212,10 @@
         <v>10</v>
       </c>
       <c r="M20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="N20" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="P20" t="b">
         <v>1</v>
@@ -1208,13 +1229,13 @@
         <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D21" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E21" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F21">
         <v>400</v>
@@ -1238,10 +1259,10 @@
         <v>25</v>
       </c>
       <c r="M21" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="N21" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="P21" t="b">
         <v>1</v>
@@ -1255,13 +1276,13 @@
         <v>10</v>
       </c>
       <c r="C22" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D22" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E22" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F22">
         <v>600</v>
@@ -1285,15 +1306,159 @@
         <v>35</v>
       </c>
       <c r="M22" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="N22" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="P22" t="b">
         <v>1</v>
       </c>
       <c r="Q22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" t="s">
+        <v>82</v>
+      </c>
+      <c r="E23" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" t="s">
+        <v>82</v>
+      </c>
+      <c r="D24" t="s">
+        <v>83</v>
+      </c>
+      <c r="E24" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" t="s">
+        <v>83</v>
+      </c>
+      <c r="D25" t="s">
+        <v>84</v>
+      </c>
+      <c r="E25" t="s">
+        <v>56</v>
+      </c>
+      <c r="F25">
+        <v>250</v>
+      </c>
+      <c r="G25" t="s">
+        <v>12</v>
+      </c>
+      <c r="H25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I25">
+        <v>600</v>
+      </c>
+      <c r="J25">
+        <v>50</v>
+      </c>
+      <c r="K25">
+        <v>5</v>
+      </c>
+      <c r="L25">
+        <v>40</v>
+      </c>
+      <c r="M25" t="s">
+        <v>65</v>
+      </c>
+      <c r="N25" t="s">
+        <v>66</v>
+      </c>
+      <c r="P25" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" t="s">
+        <v>86</v>
+      </c>
+      <c r="E26" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" t="s">
+        <v>86</v>
+      </c>
+      <c r="D27" t="s">
+        <v>87</v>
+      </c>
+      <c r="E27" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" t="s">
+        <v>87</v>
+      </c>
+      <c r="D28" t="s">
+        <v>88</v>
+      </c>
+      <c r="E28" t="s">
+        <v>56</v>
+      </c>
+      <c r="F28">
+        <v>250</v>
+      </c>
+      <c r="G28" t="s">
+        <v>12</v>
+      </c>
+      <c r="H28" t="s">
+        <v>80</v>
+      </c>
+      <c r="I28">
+        <v>600</v>
+      </c>
+      <c r="J28">
+        <v>50</v>
+      </c>
+      <c r="K28">
+        <v>5</v>
+      </c>
+      <c r="L28">
+        <v>40</v>
+      </c>
+      <c r="M28" t="s">
+        <v>65</v>
+      </c>
+      <c r="N28" t="s">
+        <v>66</v>
+      </c>
+      <c r="P28" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q28" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>